<commit_message>
Reprice Life Church tender at £50/hour labour
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016YnDZjxjEWNh6MnUGW28H9
</commit_message>
<xml_diff>
--- a/Life_Church_Tender_Hannah_Plumbing.xlsx
+++ b/Life_Church_Tender_Hannah_Plumbing.xlsx
@@ -542,11 +542,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Labour rate per operative-day (£)</t>
+          <t>Labour rate per hour (£)</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>300</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -562,11 +562,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Overheads &amp; profit on labour (%)</t>
+          <t>Extra O&amp;P on labour (%) - 0% as hourly rate is the billed rate</t>
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1314,7 +1314,7 @@
     <row r="35">
       <c r="E35" t="inlineStr">
         <is>
-          <t>Total labour days</t>
+          <t>Total labour hours</t>
         </is>
       </c>
       <c r="F35">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Labour days</t>
+          <t>Labour hours</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="D4" s="8">
         <f>C4*Tender!$D$6</f>
@@ -1442,7 +1442,7 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D5" s="8">
         <f>C5*Tender!$D$6</f>
@@ -1477,7 +1477,7 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="D6" s="8">
         <f>C6*Tender!$D$6</f>
@@ -1512,7 +1512,7 @@
         </is>
       </c>
       <c r="C7" s="11" t="n">
-        <v>0.75</v>
+        <v>6</v>
       </c>
       <c r="D7" s="8">
         <f>C7*Tender!$D$6</f>
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>0.1</v>
+        <v>0.8</v>
       </c>
       <c r="D8" s="8">
         <f>C8*Tender!$D$6</f>
@@ -1582,7 +1582,7 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>0.75</v>
+        <v>6</v>
       </c>
       <c r="D9" s="8">
         <f>C9*Tender!$D$6</f>
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>0.1</v>
+        <v>0.8</v>
       </c>
       <c r="D10" s="8">
         <f>C10*Tender!$D$6</f>
@@ -1652,7 +1652,7 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>1.25</v>
+        <v>10</v>
       </c>
       <c r="D11" s="8">
         <f>C11*Tender!$D$6</f>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="D12" s="8">
         <f>C12*Tender!$D$6</f>
@@ -1722,7 +1722,7 @@
         </is>
       </c>
       <c r="C13" s="11" t="n">
-        <v>0.1</v>
+        <v>0.8</v>
       </c>
       <c r="D13" s="8">
         <f>C13*Tender!$D$6</f>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="C14" s="11" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="D14" s="8">
         <f>C14*Tender!$D$6</f>
@@ -1792,7 +1792,7 @@
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D15" s="8">
         <f>C15*Tender!$D$6</f>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D16" s="8">
         <f>C16*Tender!$D$6</f>
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="D17" s="8">
         <f>C17*Tender!$D$6</f>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D18" s="8">
         <f>C18*Tender!$D$6</f>
@@ -1932,7 +1932,7 @@
         </is>
       </c>
       <c r="C19" s="11" t="n">
-        <v>0.75</v>
+        <v>6</v>
       </c>
       <c r="D19" s="8">
         <f>C19*Tender!$D$6</f>
@@ -1967,7 +1967,7 @@
         </is>
       </c>
       <c r="C20" s="11" t="n">
-        <v>0.75</v>
+        <v>6</v>
       </c>
       <c r="D20" s="8">
         <f>C20*Tender!$D$6</f>
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D21" s="8">
         <f>C21*Tender!$D$6</f>
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="D22" s="8">
         <f>C22*Tender!$D$6</f>
@@ -2072,7 +2072,7 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="D23" s="8">
         <f>C23*Tender!$D$6</f>
@@ -2107,7 +2107,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="D24" s="8">
         <f>C24*Tender!$D$6</f>
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="C25" s="11" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="D25" s="8">
         <f>C25*Tender!$D$6</f>

</xml_diff>